<commit_message>
Shift program +2 days: start Wed Jun 17 (Day 1 Push), end Aug 11
Groceries done Jun 15-16; training now formally starts tomorrow. All dates
in data.js and the source xlsx shifted +2 days, weekdays re-derived, week
ranges and start/end updated. Sequence unchanged (Push first).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Armen_2_Month_Gym_Meal_Plan_With_Timing.xlsx
+++ b/Armen_2_Month_Gym_Meal_Plan_With_Timing.xlsx
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="B2" s="102" t="n">
-        <v>46188</v>
+        <v>46190</v>
       </c>
       <c r="C2" s="102" t="inlineStr">
         <is>
@@ -976,7 +976,7 @@
         </is>
       </c>
       <c r="D2" s="102" t="n">
-        <v>46243</v>
+        <v>46245</v>
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
@@ -995,6 +995,7 @@
         <v>63</v>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="33" t="inlineStr">
         <is>
@@ -1177,6 +1178,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="33" t="inlineStr">
         <is>
@@ -1239,7 +1241,7 @@
       </c>
       <c r="B12" s="35" t="inlineStr">
         <is>
-          <t>Jun 15–Jun 21</t>
+          <t>Jun 17–Jun 23</t>
         </is>
       </c>
       <c r="C12" s="104" t="n">
@@ -1277,7 +1279,7 @@
       </c>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>Jun 22–Jun 28</t>
+          <t>Jun 24–Jun 30</t>
         </is>
       </c>
       <c r="C13" s="104" t="n">
@@ -1315,7 +1317,7 @@
       </c>
       <c r="B14" s="35" t="inlineStr">
         <is>
-          <t>Jun 29–Jul 05</t>
+          <t>Jul 1–Jul 7</t>
         </is>
       </c>
       <c r="C14" s="104" t="n">
@@ -1353,7 +1355,7 @@
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Jul 06–Jul 12</t>
+          <t>Jul 8–Jul 14</t>
         </is>
       </c>
       <c r="C15" s="104" t="n">
@@ -1391,7 +1393,7 @@
       </c>
       <c r="B16" s="35" t="inlineStr">
         <is>
-          <t>Jul 13–Jul 19</t>
+          <t>Jul 15–Jul 21</t>
         </is>
       </c>
       <c r="C16" s="104" t="n">
@@ -1429,7 +1431,7 @@
       </c>
       <c r="B17" s="35" t="inlineStr">
         <is>
-          <t>Jul 20–Jul 26</t>
+          <t>Jul 22–Jul 28</t>
         </is>
       </c>
       <c r="C17" s="104" t="n">
@@ -1467,7 +1469,7 @@
       </c>
       <c r="B18" s="35" t="inlineStr">
         <is>
-          <t>Jul 27–Aug 02</t>
+          <t>Jul 29–Aug 4</t>
         </is>
       </c>
       <c r="C18" s="104" t="n">
@@ -1505,7 +1507,7 @@
       </c>
       <c r="B19" s="35" t="inlineStr">
         <is>
-          <t>Aug 03–Aug 09</t>
+          <t>Aug 5–Aug 11</t>
         </is>
       </c>
       <c r="C19" s="104" t="n">
@@ -1537,6 +1539,8 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="33" t="inlineStr">
         <is>
@@ -1913,14 +1917,14 @@
     </row>
     <row r="3">
       <c r="A3" s="106" t="n">
-        <v>46188</v>
+        <v>46190</v>
       </c>
       <c r="B3" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D3" s="35" t="inlineStr">
@@ -1956,14 +1960,14 @@
     </row>
     <row r="4">
       <c r="A4" s="106" t="n">
-        <v>46189</v>
+        <v>46191</v>
       </c>
       <c r="B4" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D4" s="35" t="inlineStr">
@@ -1999,14 +2003,14 @@
     </row>
     <row r="5">
       <c r="A5" s="106" t="n">
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="B5" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D5" s="35" t="inlineStr">
@@ -2042,14 +2046,14 @@
     </row>
     <row r="6">
       <c r="A6" s="106" t="n">
-        <v>46191</v>
+        <v>46193</v>
       </c>
       <c r="B6" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D6" s="35" t="inlineStr">
@@ -2085,14 +2089,14 @@
     </row>
     <row r="7">
       <c r="A7" s="106" t="n">
-        <v>46192</v>
+        <v>46194</v>
       </c>
       <c r="B7" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D7" s="35" t="inlineStr">
@@ -2128,14 +2132,14 @@
     </row>
     <row r="8">
       <c r="A8" s="106" t="n">
-        <v>46193</v>
+        <v>46195</v>
       </c>
       <c r="B8" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D8" s="35" t="inlineStr">
@@ -2171,14 +2175,14 @@
     </row>
     <row r="9">
       <c r="A9" s="106" t="n">
-        <v>46194</v>
+        <v>46196</v>
       </c>
       <c r="B9" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D9" s="35" t="inlineStr">
@@ -2214,14 +2218,14 @@
     </row>
     <row r="10">
       <c r="A10" s="106" t="n">
-        <v>46195</v>
+        <v>46197</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D10" s="35" t="inlineStr">
@@ -2257,14 +2261,14 @@
     </row>
     <row r="11">
       <c r="A11" s="106" t="n">
-        <v>46196</v>
+        <v>46198</v>
       </c>
       <c r="B11" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D11" s="35" t="inlineStr">
@@ -2300,14 +2304,14 @@
     </row>
     <row r="12">
       <c r="A12" s="106" t="n">
-        <v>46197</v>
+        <v>46199</v>
       </c>
       <c r="B12" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D12" s="35" t="inlineStr">
@@ -2343,14 +2347,14 @@
     </row>
     <row r="13">
       <c r="A13" s="106" t="n">
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="B13" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D13" s="35" t="inlineStr">
@@ -2386,14 +2390,14 @@
     </row>
     <row r="14">
       <c r="A14" s="106" t="n">
-        <v>46199</v>
+        <v>46201</v>
       </c>
       <c r="B14" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C14" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D14" s="35" t="inlineStr">
@@ -2429,14 +2433,14 @@
     </row>
     <row r="15">
       <c r="A15" s="106" t="n">
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="B15" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D15" s="35" t="inlineStr">
@@ -2472,14 +2476,14 @@
     </row>
     <row r="16">
       <c r="A16" s="106" t="n">
-        <v>46201</v>
+        <v>46203</v>
       </c>
       <c r="B16" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D16" s="35" t="inlineStr">
@@ -2515,14 +2519,14 @@
     </row>
     <row r="17">
       <c r="A17" s="106" t="n">
-        <v>46202</v>
+        <v>46204</v>
       </c>
       <c r="B17" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D17" s="35" t="inlineStr">
@@ -2558,14 +2562,14 @@
     </row>
     <row r="18">
       <c r="A18" s="106" t="n">
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="B18" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D18" s="35" t="inlineStr">
@@ -2601,14 +2605,14 @@
     </row>
     <row r="19">
       <c r="A19" s="106" t="n">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="B19" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D19" s="35" t="inlineStr">
@@ -2644,14 +2648,14 @@
     </row>
     <row r="20">
       <c r="A20" s="106" t="n">
-        <v>46205</v>
+        <v>46207</v>
       </c>
       <c r="B20" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D20" s="35" t="inlineStr">
@@ -2687,14 +2691,14 @@
     </row>
     <row r="21">
       <c r="A21" s="106" t="n">
-        <v>46206</v>
+        <v>46208</v>
       </c>
       <c r="B21" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C21" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D21" s="35" t="inlineStr">
@@ -2730,14 +2734,14 @@
     </row>
     <row r="22">
       <c r="A22" s="106" t="n">
-        <v>46207</v>
+        <v>46209</v>
       </c>
       <c r="B22" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C22" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D22" s="35" t="inlineStr">
@@ -2773,14 +2777,14 @@
     </row>
     <row r="23">
       <c r="A23" s="106" t="n">
-        <v>46208</v>
+        <v>46210</v>
       </c>
       <c r="B23" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C23" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D23" s="35" t="inlineStr">
@@ -2816,14 +2820,14 @@
     </row>
     <row r="24">
       <c r="A24" s="106" t="n">
-        <v>46209</v>
+        <v>46211</v>
       </c>
       <c r="B24" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D24" s="35" t="inlineStr">
@@ -2859,14 +2863,14 @@
     </row>
     <row r="25">
       <c r="A25" s="106" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="B25" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C25" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D25" s="35" t="inlineStr">
@@ -2902,14 +2906,14 @@
     </row>
     <row r="26">
       <c r="A26" s="106" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="B26" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D26" s="35" t="inlineStr">
@@ -2945,14 +2949,14 @@
     </row>
     <row r="27">
       <c r="A27" s="106" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="B27" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C27" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D27" s="35" t="inlineStr">
@@ -2988,14 +2992,14 @@
     </row>
     <row r="28">
       <c r="A28" s="106" t="n">
-        <v>46213</v>
+        <v>46215</v>
       </c>
       <c r="B28" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C28" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D28" s="35" t="inlineStr">
@@ -3031,14 +3035,14 @@
     </row>
     <row r="29">
       <c r="A29" s="106" t="n">
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="B29" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C29" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D29" s="35" t="inlineStr">
@@ -3074,14 +3078,14 @@
     </row>
     <row r="30">
       <c r="A30" s="106" t="n">
-        <v>46215</v>
+        <v>46217</v>
       </c>
       <c r="B30" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C30" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D30" s="35" t="inlineStr">
@@ -3117,14 +3121,14 @@
     </row>
     <row r="31">
       <c r="A31" s="106" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="B31" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C31" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D31" s="35" t="inlineStr">
@@ -3160,14 +3164,14 @@
     </row>
     <row r="32">
       <c r="A32" s="106" t="n">
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="B32" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C32" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D32" s="35" t="inlineStr">
@@ -3203,14 +3207,14 @@
     </row>
     <row r="33">
       <c r="A33" s="106" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B33" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C33" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D33" s="35" t="inlineStr">
@@ -3246,14 +3250,14 @@
     </row>
     <row r="34">
       <c r="A34" s="106" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B34" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C34" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D34" s="35" t="inlineStr">
@@ -3289,14 +3293,14 @@
     </row>
     <row r="35">
       <c r="A35" s="106" t="n">
-        <v>46220</v>
+        <v>46222</v>
       </c>
       <c r="B35" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C35" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D35" s="35" t="inlineStr">
@@ -3332,14 +3336,14 @@
     </row>
     <row r="36">
       <c r="A36" s="106" t="n">
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="B36" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C36" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D36" s="35" t="inlineStr">
@@ -3375,14 +3379,14 @@
     </row>
     <row r="37">
       <c r="A37" s="106" t="n">
-        <v>46222</v>
+        <v>46224</v>
       </c>
       <c r="B37" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C37" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D37" s="35" t="inlineStr">
@@ -3418,14 +3422,14 @@
     </row>
     <row r="38">
       <c r="A38" s="106" t="n">
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="B38" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C38" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D38" s="35" t="inlineStr">
@@ -3461,14 +3465,14 @@
     </row>
     <row r="39">
       <c r="A39" s="106" t="n">
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="B39" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C39" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D39" s="35" t="inlineStr">
@@ -3504,14 +3508,14 @@
     </row>
     <row r="40">
       <c r="A40" s="106" t="n">
-        <v>46225</v>
+        <v>46227</v>
       </c>
       <c r="B40" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C40" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D40" s="35" t="inlineStr">
@@ -3547,14 +3551,14 @@
     </row>
     <row r="41">
       <c r="A41" s="106" t="n">
-        <v>46226</v>
+        <v>46228</v>
       </c>
       <c r="B41" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C41" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D41" s="35" t="inlineStr">
@@ -3590,14 +3594,14 @@
     </row>
     <row r="42">
       <c r="A42" s="106" t="n">
-        <v>46227</v>
+        <v>46229</v>
       </c>
       <c r="B42" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C42" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D42" s="35" t="inlineStr">
@@ -3633,14 +3637,14 @@
     </row>
     <row r="43">
       <c r="A43" s="106" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="B43" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C43" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D43" s="35" t="inlineStr">
@@ -3676,14 +3680,14 @@
     </row>
     <row r="44">
       <c r="A44" s="106" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="B44" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C44" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D44" s="35" t="inlineStr">
@@ -3719,14 +3723,14 @@
     </row>
     <row r="45">
       <c r="A45" s="106" t="n">
-        <v>46230</v>
+        <v>46232</v>
       </c>
       <c r="B45" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C45" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D45" s="35" t="inlineStr">
@@ -3762,14 +3766,14 @@
     </row>
     <row r="46">
       <c r="A46" s="106" t="n">
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="B46" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C46" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D46" s="35" t="inlineStr">
@@ -3805,14 +3809,14 @@
     </row>
     <row r="47">
       <c r="A47" s="106" t="n">
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="B47" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C47" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D47" s="35" t="inlineStr">
@@ -3848,14 +3852,14 @@
     </row>
     <row r="48">
       <c r="A48" s="106" t="n">
-        <v>46233</v>
+        <v>46235</v>
       </c>
       <c r="B48" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C48" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D48" s="35" t="inlineStr">
@@ -3891,14 +3895,14 @@
     </row>
     <row r="49">
       <c r="A49" s="106" t="n">
-        <v>46234</v>
+        <v>46236</v>
       </c>
       <c r="B49" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C49" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D49" s="35" t="inlineStr">
@@ -3934,14 +3938,14 @@
     </row>
     <row r="50">
       <c r="A50" s="106" t="n">
-        <v>46235</v>
+        <v>46237</v>
       </c>
       <c r="B50" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C50" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D50" s="35" t="inlineStr">
@@ -3977,14 +3981,14 @@
     </row>
     <row r="51">
       <c r="A51" s="106" t="n">
-        <v>46236</v>
+        <v>46238</v>
       </c>
       <c r="B51" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C51" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D51" s="35" t="inlineStr">
@@ -4020,14 +4024,14 @@
     </row>
     <row r="52">
       <c r="A52" s="106" t="n">
-        <v>46237</v>
+        <v>46239</v>
       </c>
       <c r="B52" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C52" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D52" s="35" t="inlineStr">
@@ -4063,14 +4067,14 @@
     </row>
     <row r="53">
       <c r="A53" s="106" t="n">
-        <v>46238</v>
+        <v>46240</v>
       </c>
       <c r="B53" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C53" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D53" s="35" t="inlineStr">
@@ -4106,14 +4110,14 @@
     </row>
     <row r="54">
       <c r="A54" s="106" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="B54" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C54" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D54" s="35" t="inlineStr">
@@ -4149,14 +4153,14 @@
     </row>
     <row r="55">
       <c r="A55" s="106" t="n">
-        <v>46240</v>
+        <v>46242</v>
       </c>
       <c r="B55" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C55" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D55" s="35" t="inlineStr">
@@ -4192,14 +4196,14 @@
     </row>
     <row r="56">
       <c r="A56" s="106" t="n">
-        <v>46241</v>
+        <v>46243</v>
       </c>
       <c r="B56" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C56" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D56" s="35" t="inlineStr">
@@ -4235,14 +4239,14 @@
     </row>
     <row r="57">
       <c r="A57" s="106" t="n">
-        <v>46242</v>
+        <v>46244</v>
       </c>
       <c r="B57" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C57" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D57" s="35" t="inlineStr">
@@ -4278,14 +4282,14 @@
     </row>
     <row r="58">
       <c r="A58" s="106" t="n">
-        <v>46243</v>
+        <v>46245</v>
       </c>
       <c r="B58" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C58" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D58" s="35" t="inlineStr">
@@ -6520,21 +6524,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="33" t="inlineStr">
         <is>
@@ -7446,7 +7435,7 @@
     </row>
     <row r="3">
       <c r="A3" s="106" t="n">
-        <v>46188</v>
+        <v>46190</v>
       </c>
       <c r="B3" s="35" t="n">
         <v>1</v>
@@ -7528,7 +7517,7 @@
     </row>
     <row r="4">
       <c r="A4" s="106" t="n">
-        <v>46189</v>
+        <v>46191</v>
       </c>
       <c r="B4" s="35" t="n">
         <v>1</v>
@@ -7610,7 +7599,7 @@
     </row>
     <row r="5">
       <c r="A5" s="106" t="n">
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="B5" s="35" t="n">
         <v>1</v>
@@ -7692,7 +7681,7 @@
     </row>
     <row r="6">
       <c r="A6" s="106" t="n">
-        <v>46191</v>
+        <v>46193</v>
       </c>
       <c r="B6" s="35" t="n">
         <v>1</v>
@@ -7774,7 +7763,7 @@
     </row>
     <row r="7">
       <c r="A7" s="106" t="n">
-        <v>46192</v>
+        <v>46194</v>
       </c>
       <c r="B7" s="35" t="n">
         <v>1</v>
@@ -7856,7 +7845,7 @@
     </row>
     <row r="8">
       <c r="A8" s="106" t="n">
-        <v>46193</v>
+        <v>46195</v>
       </c>
       <c r="B8" s="35" t="n">
         <v>1</v>
@@ -7942,7 +7931,7 @@
     </row>
     <row r="9">
       <c r="A9" s="106" t="n">
-        <v>46194</v>
+        <v>46196</v>
       </c>
       <c r="B9" s="35" t="n">
         <v>1</v>
@@ -8024,7 +8013,7 @@
     </row>
     <row r="10">
       <c r="A10" s="106" t="n">
-        <v>46195</v>
+        <v>46197</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>2</v>
@@ -8106,7 +8095,7 @@
     </row>
     <row r="11">
       <c r="A11" s="106" t="n">
-        <v>46196</v>
+        <v>46198</v>
       </c>
       <c r="B11" s="35" t="n">
         <v>2</v>
@@ -8188,7 +8177,7 @@
     </row>
     <row r="12">
       <c r="A12" s="106" t="n">
-        <v>46197</v>
+        <v>46199</v>
       </c>
       <c r="B12" s="35" t="n">
         <v>2</v>
@@ -8270,7 +8259,7 @@
     </row>
     <row r="13">
       <c r="A13" s="106" t="n">
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="B13" s="35" t="n">
         <v>2</v>
@@ -8352,7 +8341,7 @@
     </row>
     <row r="14">
       <c r="A14" s="106" t="n">
-        <v>46199</v>
+        <v>46201</v>
       </c>
       <c r="B14" s="35" t="n">
         <v>2</v>
@@ -8434,7 +8423,7 @@
     </row>
     <row r="15">
       <c r="A15" s="106" t="n">
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="B15" s="35" t="n">
         <v>2</v>
@@ -8520,7 +8509,7 @@
     </row>
     <row r="16">
       <c r="A16" s="106" t="n">
-        <v>46201</v>
+        <v>46203</v>
       </c>
       <c r="B16" s="35" t="n">
         <v>2</v>
@@ -8602,7 +8591,7 @@
     </row>
     <row r="17">
       <c r="A17" s="106" t="n">
-        <v>46202</v>
+        <v>46204</v>
       </c>
       <c r="B17" s="35" t="n">
         <v>3</v>
@@ -8684,7 +8673,7 @@
     </row>
     <row r="18">
       <c r="A18" s="106" t="n">
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="B18" s="35" t="n">
         <v>3</v>
@@ -8766,7 +8755,7 @@
     </row>
     <row r="19">
       <c r="A19" s="106" t="n">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="B19" s="35" t="n">
         <v>3</v>
@@ -8848,7 +8837,7 @@
     </row>
     <row r="20">
       <c r="A20" s="106" t="n">
-        <v>46205</v>
+        <v>46207</v>
       </c>
       <c r="B20" s="35" t="n">
         <v>3</v>
@@ -8930,7 +8919,7 @@
     </row>
     <row r="21">
       <c r="A21" s="106" t="n">
-        <v>46206</v>
+        <v>46208</v>
       </c>
       <c r="B21" s="35" t="n">
         <v>3</v>
@@ -9012,7 +9001,7 @@
     </row>
     <row r="22">
       <c r="A22" s="106" t="n">
-        <v>46207</v>
+        <v>46209</v>
       </c>
       <c r="B22" s="35" t="n">
         <v>3</v>
@@ -9098,7 +9087,7 @@
     </row>
     <row r="23">
       <c r="A23" s="106" t="n">
-        <v>46208</v>
+        <v>46210</v>
       </c>
       <c r="B23" s="35" t="n">
         <v>3</v>
@@ -9180,7 +9169,7 @@
     </row>
     <row r="24">
       <c r="A24" s="106" t="n">
-        <v>46209</v>
+        <v>46211</v>
       </c>
       <c r="B24" s="35" t="n">
         <v>4</v>
@@ -9262,7 +9251,7 @@
     </row>
     <row r="25">
       <c r="A25" s="106" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="B25" s="35" t="n">
         <v>4</v>
@@ -9344,7 +9333,7 @@
     </row>
     <row r="26">
       <c r="A26" s="106" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="B26" s="35" t="n">
         <v>4</v>
@@ -9426,7 +9415,7 @@
     </row>
     <row r="27">
       <c r="A27" s="106" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="B27" s="35" t="n">
         <v>4</v>
@@ -9508,7 +9497,7 @@
     </row>
     <row r="28">
       <c r="A28" s="106" t="n">
-        <v>46213</v>
+        <v>46215</v>
       </c>
       <c r="B28" s="35" t="n">
         <v>4</v>
@@ -9590,7 +9579,7 @@
     </row>
     <row r="29">
       <c r="A29" s="106" t="n">
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="B29" s="35" t="n">
         <v>4</v>
@@ -9676,7 +9665,7 @@
     </row>
     <row r="30">
       <c r="A30" s="106" t="n">
-        <v>46215</v>
+        <v>46217</v>
       </c>
       <c r="B30" s="35" t="n">
         <v>4</v>
@@ -9758,7 +9747,7 @@
     </row>
     <row r="31">
       <c r="A31" s="106" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="B31" s="35" t="n">
         <v>5</v>
@@ -9840,7 +9829,7 @@
     </row>
     <row r="32">
       <c r="A32" s="106" t="n">
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="B32" s="35" t="n">
         <v>5</v>
@@ -9922,7 +9911,7 @@
     </row>
     <row r="33">
       <c r="A33" s="106" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B33" s="35" t="n">
         <v>5</v>
@@ -10004,7 +9993,7 @@
     </row>
     <row r="34">
       <c r="A34" s="106" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B34" s="35" t="n">
         <v>5</v>
@@ -10086,7 +10075,7 @@
     </row>
     <row r="35">
       <c r="A35" s="106" t="n">
-        <v>46220</v>
+        <v>46222</v>
       </c>
       <c r="B35" s="35" t="n">
         <v>5</v>
@@ -10168,7 +10157,7 @@
     </row>
     <row r="36">
       <c r="A36" s="106" t="n">
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="B36" s="35" t="n">
         <v>5</v>
@@ -10254,7 +10243,7 @@
     </row>
     <row r="37">
       <c r="A37" s="106" t="n">
-        <v>46222</v>
+        <v>46224</v>
       </c>
       <c r="B37" s="35" t="n">
         <v>5</v>
@@ -10336,7 +10325,7 @@
     </row>
     <row r="38">
       <c r="A38" s="106" t="n">
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="B38" s="35" t="n">
         <v>6</v>
@@ -10418,7 +10407,7 @@
     </row>
     <row r="39">
       <c r="A39" s="106" t="n">
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="B39" s="35" t="n">
         <v>6</v>
@@ -10500,7 +10489,7 @@
     </row>
     <row r="40">
       <c r="A40" s="106" t="n">
-        <v>46225</v>
+        <v>46227</v>
       </c>
       <c r="B40" s="35" t="n">
         <v>6</v>
@@ -10582,7 +10571,7 @@
     </row>
     <row r="41">
       <c r="A41" s="106" t="n">
-        <v>46226</v>
+        <v>46228</v>
       </c>
       <c r="B41" s="35" t="n">
         <v>6</v>
@@ -10664,7 +10653,7 @@
     </row>
     <row r="42">
       <c r="A42" s="106" t="n">
-        <v>46227</v>
+        <v>46229</v>
       </c>
       <c r="B42" s="35" t="n">
         <v>6</v>
@@ -10746,7 +10735,7 @@
     </row>
     <row r="43">
       <c r="A43" s="106" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="B43" s="35" t="n">
         <v>6</v>
@@ -10832,7 +10821,7 @@
     </row>
     <row r="44">
       <c r="A44" s="106" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="B44" s="35" t="n">
         <v>6</v>
@@ -10914,7 +10903,7 @@
     </row>
     <row r="45">
       <c r="A45" s="106" t="n">
-        <v>46230</v>
+        <v>46232</v>
       </c>
       <c r="B45" s="35" t="n">
         <v>7</v>
@@ -10996,7 +10985,7 @@
     </row>
     <row r="46">
       <c r="A46" s="106" t="n">
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="B46" s="35" t="n">
         <v>7</v>
@@ -11078,7 +11067,7 @@
     </row>
     <row r="47">
       <c r="A47" s="106" t="n">
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="B47" s="35" t="n">
         <v>7</v>
@@ -11160,7 +11149,7 @@
     </row>
     <row r="48">
       <c r="A48" s="106" t="n">
-        <v>46233</v>
+        <v>46235</v>
       </c>
       <c r="B48" s="35" t="n">
         <v>7</v>
@@ -11242,7 +11231,7 @@
     </row>
     <row r="49">
       <c r="A49" s="106" t="n">
-        <v>46234</v>
+        <v>46236</v>
       </c>
       <c r="B49" s="35" t="n">
         <v>7</v>
@@ -11324,7 +11313,7 @@
     </row>
     <row r="50">
       <c r="A50" s="106" t="n">
-        <v>46235</v>
+        <v>46237</v>
       </c>
       <c r="B50" s="35" t="n">
         <v>7</v>
@@ -11410,7 +11399,7 @@
     </row>
     <row r="51">
       <c r="A51" s="106" t="n">
-        <v>46236</v>
+        <v>46238</v>
       </c>
       <c r="B51" s="35" t="n">
         <v>7</v>
@@ -11492,7 +11481,7 @@
     </row>
     <row r="52">
       <c r="A52" s="106" t="n">
-        <v>46237</v>
+        <v>46239</v>
       </c>
       <c r="B52" s="35" t="n">
         <v>8</v>
@@ -11574,7 +11563,7 @@
     </row>
     <row r="53">
       <c r="A53" s="106" t="n">
-        <v>46238</v>
+        <v>46240</v>
       </c>
       <c r="B53" s="35" t="n">
         <v>8</v>
@@ -11656,7 +11645,7 @@
     </row>
     <row r="54">
       <c r="A54" s="106" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="B54" s="35" t="n">
         <v>8</v>
@@ -11738,7 +11727,7 @@
     </row>
     <row r="55">
       <c r="A55" s="106" t="n">
-        <v>46240</v>
+        <v>46242</v>
       </c>
       <c r="B55" s="35" t="n">
         <v>8</v>
@@ -11820,7 +11809,7 @@
     </row>
     <row r="56">
       <c r="A56" s="106" t="n">
-        <v>46241</v>
+        <v>46243</v>
       </c>
       <c r="B56" s="35" t="n">
         <v>8</v>
@@ -11902,7 +11891,7 @@
     </row>
     <row r="57">
       <c r="A57" s="106" t="n">
-        <v>46242</v>
+        <v>46244</v>
       </c>
       <c r="B57" s="35" t="n">
         <v>8</v>
@@ -11988,7 +11977,7 @@
     </row>
     <row r="58">
       <c r="A58" s="106" t="n">
-        <v>46243</v>
+        <v>46245</v>
       </c>
       <c r="B58" s="35" t="n">
         <v>8</v>
@@ -13541,11 +13530,11 @@
     </row>
     <row r="3">
       <c r="A3" s="106" t="n">
-        <v>46188</v>
+        <v>46190</v>
       </c>
       <c r="B3" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C3" s="104" t="str"/>
@@ -13568,11 +13557,11 @@
     </row>
     <row r="4">
       <c r="A4" s="106" t="n">
-        <v>46189</v>
+        <v>46191</v>
       </c>
       <c r="B4" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C4" s="104" t="str"/>
@@ -13595,11 +13584,11 @@
     </row>
     <row r="5">
       <c r="A5" s="106" t="n">
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="B5" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C5" s="104" t="str"/>
@@ -13622,11 +13611,11 @@
     </row>
     <row r="6">
       <c r="A6" s="106" t="n">
-        <v>46191</v>
+        <v>46193</v>
       </c>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C6" s="104" t="str"/>
@@ -13649,11 +13638,11 @@
     </row>
     <row r="7">
       <c r="A7" s="106" t="n">
-        <v>46192</v>
+        <v>46194</v>
       </c>
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C7" s="104" t="str"/>
@@ -13676,11 +13665,11 @@
     </row>
     <row r="8">
       <c r="A8" s="106" t="n">
-        <v>46193</v>
+        <v>46195</v>
       </c>
       <c r="B8" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C8" s="104" t="str"/>
@@ -13703,11 +13692,11 @@
     </row>
     <row r="9">
       <c r="A9" s="106" t="n">
-        <v>46194</v>
+        <v>46196</v>
       </c>
       <c r="B9" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C9" s="104" t="str"/>
@@ -13730,11 +13719,11 @@
     </row>
     <row r="10">
       <c r="A10" s="106" t="n">
-        <v>46195</v>
+        <v>46197</v>
       </c>
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C10" s="104" t="str"/>
@@ -13757,11 +13746,11 @@
     </row>
     <row r="11">
       <c r="A11" s="106" t="n">
-        <v>46196</v>
+        <v>46198</v>
       </c>
       <c r="B11" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C11" s="104" t="str"/>
@@ -13784,11 +13773,11 @@
     </row>
     <row r="12">
       <c r="A12" s="106" t="n">
-        <v>46197</v>
+        <v>46199</v>
       </c>
       <c r="B12" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C12" s="104" t="str"/>
@@ -13811,11 +13800,11 @@
     </row>
     <row r="13">
       <c r="A13" s="106" t="n">
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C13" s="104" t="str"/>
@@ -13838,11 +13827,11 @@
     </row>
     <row r="14">
       <c r="A14" s="106" t="n">
-        <v>46199</v>
+        <v>46201</v>
       </c>
       <c r="B14" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C14" s="104" t="str"/>
@@ -13865,11 +13854,11 @@
     </row>
     <row r="15">
       <c r="A15" s="106" t="n">
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C15" s="104" t="str"/>
@@ -13892,11 +13881,11 @@
     </row>
     <row r="16">
       <c r="A16" s="106" t="n">
-        <v>46201</v>
+        <v>46203</v>
       </c>
       <c r="B16" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C16" s="104" t="str"/>
@@ -13919,11 +13908,11 @@
     </row>
     <row r="17">
       <c r="A17" s="106" t="n">
-        <v>46202</v>
+        <v>46204</v>
       </c>
       <c r="B17" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C17" s="104" t="str"/>
@@ -13946,11 +13935,11 @@
     </row>
     <row r="18">
       <c r="A18" s="106" t="n">
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="B18" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C18" s="104" t="str"/>
@@ -13973,11 +13962,11 @@
     </row>
     <row r="19">
       <c r="A19" s="106" t="n">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="B19" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C19" s="104" t="str"/>
@@ -14000,11 +13989,11 @@
     </row>
     <row r="20">
       <c r="A20" s="106" t="n">
-        <v>46205</v>
+        <v>46207</v>
       </c>
       <c r="B20" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C20" s="104" t="str"/>
@@ -14027,11 +14016,11 @@
     </row>
     <row r="21">
       <c r="A21" s="106" t="n">
-        <v>46206</v>
+        <v>46208</v>
       </c>
       <c r="B21" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C21" s="104" t="str"/>
@@ -14054,11 +14043,11 @@
     </row>
     <row r="22">
       <c r="A22" s="106" t="n">
-        <v>46207</v>
+        <v>46209</v>
       </c>
       <c r="B22" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C22" s="104" t="str"/>
@@ -14081,11 +14070,11 @@
     </row>
     <row r="23">
       <c r="A23" s="106" t="n">
-        <v>46208</v>
+        <v>46210</v>
       </c>
       <c r="B23" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C23" s="104" t="str"/>
@@ -14108,11 +14097,11 @@
     </row>
     <row r="24">
       <c r="A24" s="106" t="n">
-        <v>46209</v>
+        <v>46211</v>
       </c>
       <c r="B24" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C24" s="104" t="str"/>
@@ -14135,11 +14124,11 @@
     </row>
     <row r="25">
       <c r="A25" s="106" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="B25" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C25" s="104" t="str"/>
@@ -14162,11 +14151,11 @@
     </row>
     <row r="26">
       <c r="A26" s="106" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="B26" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C26" s="104" t="str"/>
@@ -14189,11 +14178,11 @@
     </row>
     <row r="27">
       <c r="A27" s="106" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="B27" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C27" s="104" t="str"/>
@@ -14216,11 +14205,11 @@
     </row>
     <row r="28">
       <c r="A28" s="106" t="n">
-        <v>46213</v>
+        <v>46215</v>
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C28" s="104" t="str"/>
@@ -14243,11 +14232,11 @@
     </row>
     <row r="29">
       <c r="A29" s="106" t="n">
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="B29" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C29" s="104" t="str"/>
@@ -14270,11 +14259,11 @@
     </row>
     <row r="30">
       <c r="A30" s="106" t="n">
-        <v>46215</v>
+        <v>46217</v>
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C30" s="104" t="str"/>
@@ -14297,11 +14286,11 @@
     </row>
     <row r="31">
       <c r="A31" s="106" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C31" s="104" t="str"/>
@@ -14324,11 +14313,11 @@
     </row>
     <row r="32">
       <c r="A32" s="106" t="n">
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C32" s="104" t="str"/>
@@ -14351,11 +14340,11 @@
     </row>
     <row r="33">
       <c r="A33" s="106" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C33" s="104" t="str"/>
@@ -14378,11 +14367,11 @@
     </row>
     <row r="34">
       <c r="A34" s="106" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C34" s="104" t="str"/>
@@ -14405,11 +14394,11 @@
     </row>
     <row r="35">
       <c r="A35" s="106" t="n">
-        <v>46220</v>
+        <v>46222</v>
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C35" s="104" t="str"/>
@@ -14432,11 +14421,11 @@
     </row>
     <row r="36">
       <c r="A36" s="106" t="n">
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C36" s="104" t="str"/>
@@ -14459,11 +14448,11 @@
     </row>
     <row r="37">
       <c r="A37" s="106" t="n">
-        <v>46222</v>
+        <v>46224</v>
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C37" s="104" t="str"/>
@@ -14486,11 +14475,11 @@
     </row>
     <row r="38">
       <c r="A38" s="106" t="n">
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C38" s="104" t="str"/>
@@ -14513,11 +14502,11 @@
     </row>
     <row r="39">
       <c r="A39" s="106" t="n">
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C39" s="104" t="str"/>
@@ -14540,11 +14529,11 @@
     </row>
     <row r="40">
       <c r="A40" s="106" t="n">
-        <v>46225</v>
+        <v>46227</v>
       </c>
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C40" s="104" t="str"/>
@@ -14567,11 +14556,11 @@
     </row>
     <row r="41">
       <c r="A41" s="106" t="n">
-        <v>46226</v>
+        <v>46228</v>
       </c>
       <c r="B41" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C41" s="104" t="str"/>
@@ -14594,11 +14583,11 @@
     </row>
     <row r="42">
       <c r="A42" s="106" t="n">
-        <v>46227</v>
+        <v>46229</v>
       </c>
       <c r="B42" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C42" s="104" t="str"/>
@@ -14621,11 +14610,11 @@
     </row>
     <row r="43">
       <c r="A43" s="106" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="B43" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C43" s="104" t="str"/>
@@ -14648,11 +14637,11 @@
     </row>
     <row r="44">
       <c r="A44" s="106" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="B44" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C44" s="104" t="str"/>
@@ -14675,11 +14664,11 @@
     </row>
     <row r="45">
       <c r="A45" s="106" t="n">
-        <v>46230</v>
+        <v>46232</v>
       </c>
       <c r="B45" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C45" s="104" t="str"/>
@@ -14702,11 +14691,11 @@
     </row>
     <row r="46">
       <c r="A46" s="106" t="n">
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="B46" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C46" s="104" t="str"/>
@@ -14729,11 +14718,11 @@
     </row>
     <row r="47">
       <c r="A47" s="106" t="n">
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="B47" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C47" s="104" t="str"/>
@@ -14756,11 +14745,11 @@
     </row>
     <row r="48">
       <c r="A48" s="106" t="n">
-        <v>46233</v>
+        <v>46235</v>
       </c>
       <c r="B48" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C48" s="104" t="str"/>
@@ -14783,11 +14772,11 @@
     </row>
     <row r="49">
       <c r="A49" s="106" t="n">
-        <v>46234</v>
+        <v>46236</v>
       </c>
       <c r="B49" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C49" s="104" t="str"/>
@@ -14810,11 +14799,11 @@
     </row>
     <row r="50">
       <c r="A50" s="106" t="n">
-        <v>46235</v>
+        <v>46237</v>
       </c>
       <c r="B50" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C50" s="104" t="str"/>
@@ -14837,11 +14826,11 @@
     </row>
     <row r="51">
       <c r="A51" s="106" t="n">
-        <v>46236</v>
+        <v>46238</v>
       </c>
       <c r="B51" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C51" s="104" t="str"/>
@@ -14864,11 +14853,11 @@
     </row>
     <row r="52">
       <c r="A52" s="106" t="n">
-        <v>46237</v>
+        <v>46239</v>
       </c>
       <c r="B52" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C52" s="104" t="str"/>
@@ -14891,11 +14880,11 @@
     </row>
     <row r="53">
       <c r="A53" s="106" t="n">
-        <v>46238</v>
+        <v>46240</v>
       </c>
       <c r="B53" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C53" s="104" t="str"/>
@@ -14918,11 +14907,11 @@
     </row>
     <row r="54">
       <c r="A54" s="106" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="B54" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C54" s="104" t="str"/>
@@ -14945,11 +14934,11 @@
     </row>
     <row r="55">
       <c r="A55" s="106" t="n">
-        <v>46240</v>
+        <v>46242</v>
       </c>
       <c r="B55" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C55" s="104" t="str"/>
@@ -14972,11 +14961,11 @@
     </row>
     <row r="56">
       <c r="A56" s="106" t="n">
-        <v>46241</v>
+        <v>46243</v>
       </c>
       <c r="B56" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C56" s="104" t="str"/>
@@ -14999,11 +14988,11 @@
     </row>
     <row r="57">
       <c r="A57" s="106" t="n">
-        <v>46242</v>
+        <v>46244</v>
       </c>
       <c r="B57" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C57" s="104" t="str"/>
@@ -15026,11 +15015,11 @@
     </row>
     <row r="58">
       <c r="A58" s="106" t="n">
-        <v>46243</v>
+        <v>46245</v>
       </c>
       <c r="B58" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C58" s="104" t="str"/>

</xml_diff>

<commit_message>
Re-shift program -1 day: Day 1 (Push) = Tue Jun 16, today is Day 2 (Pull)
Corrected the start: groceries were Jun 15, first workout (Push) was done
Jun 16. Start now Jun 16, ends Aug 10. Yesterday is in-plan, so it's
navigable on the Today screen for marking meals/weights.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Armen_2_Month_Gym_Meal_Plan_With_Timing.xlsx
+++ b/Armen_2_Month_Gym_Meal_Plan_With_Timing.xlsx
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="B2" s="102" t="n">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="C2" s="102" t="inlineStr">
         <is>
@@ -976,7 +976,7 @@
         </is>
       </c>
       <c r="D2" s="102" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B12" s="35" t="inlineStr">
         <is>
-          <t>Jun 17–Jun 23</t>
+          <t>Jun 16–Jun 22</t>
         </is>
       </c>
       <c r="C12" s="104" t="n">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>Jun 24–Jun 30</t>
+          <t>Jun 23–Jun 29</t>
         </is>
       </c>
       <c r="C13" s="104" t="n">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B14" s="35" t="inlineStr">
         <is>
-          <t>Jul 1–Jul 7</t>
+          <t>Jun 30–Jul 6</t>
         </is>
       </c>
       <c r="C14" s="104" t="n">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Jul 8–Jul 14</t>
+          <t>Jul 7–Jul 13</t>
         </is>
       </c>
       <c r="C15" s="104" t="n">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B16" s="35" t="inlineStr">
         <is>
-          <t>Jul 15–Jul 21</t>
+          <t>Jul 14–Jul 20</t>
         </is>
       </c>
       <c r="C16" s="104" t="n">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B17" s="35" t="inlineStr">
         <is>
-          <t>Jul 22–Jul 28</t>
+          <t>Jul 21–Jul 27</t>
         </is>
       </c>
       <c r="C17" s="104" t="n">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="B18" s="35" t="inlineStr">
         <is>
-          <t>Jul 29–Aug 4</t>
+          <t>Jul 28–Aug 3</t>
         </is>
       </c>
       <c r="C18" s="104" t="n">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="B19" s="35" t="inlineStr">
         <is>
-          <t>Aug 5–Aug 11</t>
+          <t>Aug 4–Aug 10</t>
         </is>
       </c>
       <c r="C19" s="104" t="n">
@@ -1917,14 +1917,14 @@
     </row>
     <row r="3">
       <c r="A3" s="106" t="n">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="B3" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D3" s="35" t="inlineStr">
@@ -1960,14 +1960,14 @@
     </row>
     <row r="4">
       <c r="A4" s="106" t="n">
-        <v>46191</v>
+        <v>46190</v>
       </c>
       <c r="B4" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D4" s="35" t="inlineStr">
@@ -2003,14 +2003,14 @@
     </row>
     <row r="5">
       <c r="A5" s="106" t="n">
-        <v>46192</v>
+        <v>46191</v>
       </c>
       <c r="B5" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D5" s="35" t="inlineStr">
@@ -2046,14 +2046,14 @@
     </row>
     <row r="6">
       <c r="A6" s="106" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B6" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D6" s="35" t="inlineStr">
@@ -2089,14 +2089,14 @@
     </row>
     <row r="7">
       <c r="A7" s="106" t="n">
-        <v>46194</v>
+        <v>46193</v>
       </c>
       <c r="B7" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D7" s="35" t="inlineStr">
@@ -2132,14 +2132,14 @@
     </row>
     <row r="8">
       <c r="A8" s="106" t="n">
-        <v>46195</v>
+        <v>46194</v>
       </c>
       <c r="B8" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D8" s="35" t="inlineStr">
@@ -2175,14 +2175,14 @@
     </row>
     <row r="9">
       <c r="A9" s="106" t="n">
-        <v>46196</v>
+        <v>46195</v>
       </c>
       <c r="B9" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D9" s="35" t="inlineStr">
@@ -2218,14 +2218,14 @@
     </row>
     <row r="10">
       <c r="A10" s="106" t="n">
-        <v>46197</v>
+        <v>46196</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D10" s="35" t="inlineStr">
@@ -2261,14 +2261,14 @@
     </row>
     <row r="11">
       <c r="A11" s="106" t="n">
-        <v>46198</v>
+        <v>46197</v>
       </c>
       <c r="B11" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D11" s="35" t="inlineStr">
@@ -2304,14 +2304,14 @@
     </row>
     <row r="12">
       <c r="A12" s="106" t="n">
-        <v>46199</v>
+        <v>46198</v>
       </c>
       <c r="B12" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D12" s="35" t="inlineStr">
@@ -2347,14 +2347,14 @@
     </row>
     <row r="13">
       <c r="A13" s="106" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B13" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D13" s="35" t="inlineStr">
@@ -2390,14 +2390,14 @@
     </row>
     <row r="14">
       <c r="A14" s="106" t="n">
-        <v>46201</v>
+        <v>46200</v>
       </c>
       <c r="B14" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C14" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D14" s="35" t="inlineStr">
@@ -2433,14 +2433,14 @@
     </row>
     <row r="15">
       <c r="A15" s="106" t="n">
-        <v>46202</v>
+        <v>46201</v>
       </c>
       <c r="B15" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D15" s="35" t="inlineStr">
@@ -2476,14 +2476,14 @@
     </row>
     <row r="16">
       <c r="A16" s="106" t="n">
-        <v>46203</v>
+        <v>46202</v>
       </c>
       <c r="B16" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D16" s="35" t="inlineStr">
@@ -2519,14 +2519,14 @@
     </row>
     <row r="17">
       <c r="A17" s="106" t="n">
-        <v>46204</v>
+        <v>46203</v>
       </c>
       <c r="B17" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D17" s="35" t="inlineStr">
@@ -2562,14 +2562,14 @@
     </row>
     <row r="18">
       <c r="A18" s="106" t="n">
-        <v>46205</v>
+        <v>46204</v>
       </c>
       <c r="B18" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D18" s="35" t="inlineStr">
@@ -2605,14 +2605,14 @@
     </row>
     <row r="19">
       <c r="A19" s="106" t="n">
-        <v>46206</v>
+        <v>46205</v>
       </c>
       <c r="B19" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D19" s="35" t="inlineStr">
@@ -2648,14 +2648,14 @@
     </row>
     <row r="20">
       <c r="A20" s="106" t="n">
-        <v>46207</v>
+        <v>46206</v>
       </c>
       <c r="B20" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D20" s="35" t="inlineStr">
@@ -2691,14 +2691,14 @@
     </row>
     <row r="21">
       <c r="A21" s="106" t="n">
-        <v>46208</v>
+        <v>46207</v>
       </c>
       <c r="B21" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C21" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D21" s="35" t="inlineStr">
@@ -2734,14 +2734,14 @@
     </row>
     <row r="22">
       <c r="A22" s="106" t="n">
-        <v>46209</v>
+        <v>46208</v>
       </c>
       <c r="B22" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C22" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D22" s="35" t="inlineStr">
@@ -2777,14 +2777,14 @@
     </row>
     <row r="23">
       <c r="A23" s="106" t="n">
-        <v>46210</v>
+        <v>46209</v>
       </c>
       <c r="B23" s="35" t="n">
         <v>3</v>
       </c>
       <c r="C23" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D23" s="35" t="inlineStr">
@@ -2820,14 +2820,14 @@
     </row>
     <row r="24">
       <c r="A24" s="106" t="n">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="B24" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D24" s="35" t="inlineStr">
@@ -2863,14 +2863,14 @@
     </row>
     <row r="25">
       <c r="A25" s="106" t="n">
-        <v>46212</v>
+        <v>46211</v>
       </c>
       <c r="B25" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C25" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D25" s="35" t="inlineStr">
@@ -2906,14 +2906,14 @@
     </row>
     <row r="26">
       <c r="A26" s="106" t="n">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="B26" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D26" s="35" t="inlineStr">
@@ -2949,14 +2949,14 @@
     </row>
     <row r="27">
       <c r="A27" s="106" t="n">
-        <v>46214</v>
+        <v>46213</v>
       </c>
       <c r="B27" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C27" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D27" s="35" t="inlineStr">
@@ -2992,14 +2992,14 @@
     </row>
     <row r="28">
       <c r="A28" s="106" t="n">
-        <v>46215</v>
+        <v>46214</v>
       </c>
       <c r="B28" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C28" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D28" s="35" t="inlineStr">
@@ -3035,14 +3035,14 @@
     </row>
     <row r="29">
       <c r="A29" s="106" t="n">
-        <v>46216</v>
+        <v>46215</v>
       </c>
       <c r="B29" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C29" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D29" s="35" t="inlineStr">
@@ -3078,14 +3078,14 @@
     </row>
     <row r="30">
       <c r="A30" s="106" t="n">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="B30" s="35" t="n">
         <v>4</v>
       </c>
       <c r="C30" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D30" s="35" t="inlineStr">
@@ -3121,14 +3121,14 @@
     </row>
     <row r="31">
       <c r="A31" s="106" t="n">
-        <v>46218</v>
+        <v>46217</v>
       </c>
       <c r="B31" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C31" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D31" s="35" t="inlineStr">
@@ -3164,14 +3164,14 @@
     </row>
     <row r="32">
       <c r="A32" s="106" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="B32" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C32" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D32" s="35" t="inlineStr">
@@ -3207,14 +3207,14 @@
     </row>
     <row r="33">
       <c r="A33" s="106" t="n">
-        <v>46220</v>
+        <v>46219</v>
       </c>
       <c r="B33" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C33" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D33" s="35" t="inlineStr">
@@ -3250,14 +3250,14 @@
     </row>
     <row r="34">
       <c r="A34" s="106" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="B34" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C34" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D34" s="35" t="inlineStr">
@@ -3293,14 +3293,14 @@
     </row>
     <row r="35">
       <c r="A35" s="106" t="n">
-        <v>46222</v>
+        <v>46221</v>
       </c>
       <c r="B35" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C35" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D35" s="35" t="inlineStr">
@@ -3336,14 +3336,14 @@
     </row>
     <row r="36">
       <c r="A36" s="106" t="n">
-        <v>46223</v>
+        <v>46222</v>
       </c>
       <c r="B36" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C36" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D36" s="35" t="inlineStr">
@@ -3379,14 +3379,14 @@
     </row>
     <row r="37">
       <c r="A37" s="106" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="B37" s="35" t="n">
         <v>5</v>
       </c>
       <c r="C37" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D37" s="35" t="inlineStr">
@@ -3422,14 +3422,14 @@
     </row>
     <row r="38">
       <c r="A38" s="106" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="B38" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C38" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D38" s="35" t="inlineStr">
@@ -3465,14 +3465,14 @@
     </row>
     <row r="39">
       <c r="A39" s="106" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="B39" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C39" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D39" s="35" t="inlineStr">
@@ -3508,14 +3508,14 @@
     </row>
     <row r="40">
       <c r="A40" s="106" t="n">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="B40" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C40" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D40" s="35" t="inlineStr">
@@ -3551,14 +3551,14 @@
     </row>
     <row r="41">
       <c r="A41" s="106" t="n">
-        <v>46228</v>
+        <v>46227</v>
       </c>
       <c r="B41" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C41" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D41" s="35" t="inlineStr">
@@ -3594,14 +3594,14 @@
     </row>
     <row r="42">
       <c r="A42" s="106" t="n">
-        <v>46229</v>
+        <v>46228</v>
       </c>
       <c r="B42" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C42" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D42" s="35" t="inlineStr">
@@ -3637,14 +3637,14 @@
     </row>
     <row r="43">
       <c r="A43" s="106" t="n">
-        <v>46230</v>
+        <v>46229</v>
       </c>
       <c r="B43" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C43" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D43" s="35" t="inlineStr">
@@ -3680,14 +3680,14 @@
     </row>
     <row r="44">
       <c r="A44" s="106" t="n">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="B44" s="35" t="n">
         <v>6</v>
       </c>
       <c r="C44" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D44" s="35" t="inlineStr">
@@ -3723,14 +3723,14 @@
     </row>
     <row r="45">
       <c r="A45" s="106" t="n">
-        <v>46232</v>
+        <v>46231</v>
       </c>
       <c r="B45" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C45" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D45" s="35" t="inlineStr">
@@ -3766,14 +3766,14 @@
     </row>
     <row r="46">
       <c r="A46" s="106" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="B46" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C46" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D46" s="35" t="inlineStr">
@@ -3809,14 +3809,14 @@
     </row>
     <row r="47">
       <c r="A47" s="106" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="B47" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C47" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D47" s="35" t="inlineStr">
@@ -3852,14 +3852,14 @@
     </row>
     <row r="48">
       <c r="A48" s="106" t="n">
-        <v>46235</v>
+        <v>46234</v>
       </c>
       <c r="B48" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C48" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D48" s="35" t="inlineStr">
@@ -3895,14 +3895,14 @@
     </row>
     <row r="49">
       <c r="A49" s="106" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B49" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C49" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D49" s="35" t="inlineStr">
@@ -3938,14 +3938,14 @@
     </row>
     <row r="50">
       <c r="A50" s="106" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B50" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C50" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D50" s="35" t="inlineStr">
@@ -3981,14 +3981,14 @@
     </row>
     <row r="51">
       <c r="A51" s="106" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="B51" s="35" t="n">
         <v>7</v>
       </c>
       <c r="C51" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D51" s="35" t="inlineStr">
@@ -4024,14 +4024,14 @@
     </row>
     <row r="52">
       <c r="A52" s="106" t="n">
-        <v>46239</v>
+        <v>46238</v>
       </c>
       <c r="B52" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C52" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D52" s="35" t="inlineStr">
@@ -4067,14 +4067,14 @@
     </row>
     <row r="53">
       <c r="A53" s="106" t="n">
-        <v>46240</v>
+        <v>46239</v>
       </c>
       <c r="B53" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C53" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D53" s="35" t="inlineStr">
@@ -4110,14 +4110,14 @@
     </row>
     <row r="54">
       <c r="A54" s="106" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="B54" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C54" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D54" s="35" t="inlineStr">
@@ -4153,14 +4153,14 @@
     </row>
     <row r="55">
       <c r="A55" s="106" t="n">
-        <v>46242</v>
+        <v>46241</v>
       </c>
       <c r="B55" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C55" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="D55" s="35" t="inlineStr">
@@ -4196,14 +4196,14 @@
     </row>
     <row r="56">
       <c r="A56" s="106" t="n">
-        <v>46243</v>
+        <v>46242</v>
       </c>
       <c r="B56" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C56" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D56" s="35" t="inlineStr">
@@ -4239,14 +4239,14 @@
     </row>
     <row r="57">
       <c r="A57" s="106" t="n">
-        <v>46244</v>
+        <v>46243</v>
       </c>
       <c r="B57" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C57" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="D57" s="35" t="inlineStr">
@@ -4282,14 +4282,14 @@
     </row>
     <row r="58">
       <c r="A58" s="106" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="B58" s="35" t="n">
         <v>8</v>
       </c>
       <c r="C58" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="D58" s="35" t="inlineStr">
@@ -7435,7 +7435,7 @@
     </row>
     <row r="3">
       <c r="A3" s="106" t="n">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="B3" s="35" t="n">
         <v>1</v>
@@ -7517,7 +7517,7 @@
     </row>
     <row r="4">
       <c r="A4" s="106" t="n">
-        <v>46191</v>
+        <v>46190</v>
       </c>
       <c r="B4" s="35" t="n">
         <v>1</v>
@@ -7599,7 +7599,7 @@
     </row>
     <row r="5">
       <c r="A5" s="106" t="n">
-        <v>46192</v>
+        <v>46191</v>
       </c>
       <c r="B5" s="35" t="n">
         <v>1</v>
@@ -7681,7 +7681,7 @@
     </row>
     <row r="6">
       <c r="A6" s="106" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B6" s="35" t="n">
         <v>1</v>
@@ -7763,7 +7763,7 @@
     </row>
     <row r="7">
       <c r="A7" s="106" t="n">
-        <v>46194</v>
+        <v>46193</v>
       </c>
       <c r="B7" s="35" t="n">
         <v>1</v>
@@ -7845,7 +7845,7 @@
     </row>
     <row r="8">
       <c r="A8" s="106" t="n">
-        <v>46195</v>
+        <v>46194</v>
       </c>
       <c r="B8" s="35" t="n">
         <v>1</v>
@@ -7931,7 +7931,7 @@
     </row>
     <row r="9">
       <c r="A9" s="106" t="n">
-        <v>46196</v>
+        <v>46195</v>
       </c>
       <c r="B9" s="35" t="n">
         <v>1</v>
@@ -8013,7 +8013,7 @@
     </row>
     <row r="10">
       <c r="A10" s="106" t="n">
-        <v>46197</v>
+        <v>46196</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>2</v>
@@ -8095,7 +8095,7 @@
     </row>
     <row r="11">
       <c r="A11" s="106" t="n">
-        <v>46198</v>
+        <v>46197</v>
       </c>
       <c r="B11" s="35" t="n">
         <v>2</v>
@@ -8177,7 +8177,7 @@
     </row>
     <row r="12">
       <c r="A12" s="106" t="n">
-        <v>46199</v>
+        <v>46198</v>
       </c>
       <c r="B12" s="35" t="n">
         <v>2</v>
@@ -8259,7 +8259,7 @@
     </row>
     <row r="13">
       <c r="A13" s="106" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B13" s="35" t="n">
         <v>2</v>
@@ -8341,7 +8341,7 @@
     </row>
     <row r="14">
       <c r="A14" s="106" t="n">
-        <v>46201</v>
+        <v>46200</v>
       </c>
       <c r="B14" s="35" t="n">
         <v>2</v>
@@ -8423,7 +8423,7 @@
     </row>
     <row r="15">
       <c r="A15" s="106" t="n">
-        <v>46202</v>
+        <v>46201</v>
       </c>
       <c r="B15" s="35" t="n">
         <v>2</v>
@@ -8509,7 +8509,7 @@
     </row>
     <row r="16">
       <c r="A16" s="106" t="n">
-        <v>46203</v>
+        <v>46202</v>
       </c>
       <c r="B16" s="35" t="n">
         <v>2</v>
@@ -8591,7 +8591,7 @@
     </row>
     <row r="17">
       <c r="A17" s="106" t="n">
-        <v>46204</v>
+        <v>46203</v>
       </c>
       <c r="B17" s="35" t="n">
         <v>3</v>
@@ -8673,7 +8673,7 @@
     </row>
     <row r="18">
       <c r="A18" s="106" t="n">
-        <v>46205</v>
+        <v>46204</v>
       </c>
       <c r="B18" s="35" t="n">
         <v>3</v>
@@ -8755,7 +8755,7 @@
     </row>
     <row r="19">
       <c r="A19" s="106" t="n">
-        <v>46206</v>
+        <v>46205</v>
       </c>
       <c r="B19" s="35" t="n">
         <v>3</v>
@@ -8837,7 +8837,7 @@
     </row>
     <row r="20">
       <c r="A20" s="106" t="n">
-        <v>46207</v>
+        <v>46206</v>
       </c>
       <c r="B20" s="35" t="n">
         <v>3</v>
@@ -8919,7 +8919,7 @@
     </row>
     <row r="21">
       <c r="A21" s="106" t="n">
-        <v>46208</v>
+        <v>46207</v>
       </c>
       <c r="B21" s="35" t="n">
         <v>3</v>
@@ -9001,7 +9001,7 @@
     </row>
     <row r="22">
       <c r="A22" s="106" t="n">
-        <v>46209</v>
+        <v>46208</v>
       </c>
       <c r="B22" s="35" t="n">
         <v>3</v>
@@ -9087,7 +9087,7 @@
     </row>
     <row r="23">
       <c r="A23" s="106" t="n">
-        <v>46210</v>
+        <v>46209</v>
       </c>
       <c r="B23" s="35" t="n">
         <v>3</v>
@@ -9169,7 +9169,7 @@
     </row>
     <row r="24">
       <c r="A24" s="106" t="n">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="B24" s="35" t="n">
         <v>4</v>
@@ -9251,7 +9251,7 @@
     </row>
     <row r="25">
       <c r="A25" s="106" t="n">
-        <v>46212</v>
+        <v>46211</v>
       </c>
       <c r="B25" s="35" t="n">
         <v>4</v>
@@ -9333,7 +9333,7 @@
     </row>
     <row r="26">
       <c r="A26" s="106" t="n">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="B26" s="35" t="n">
         <v>4</v>
@@ -9415,7 +9415,7 @@
     </row>
     <row r="27">
       <c r="A27" s="106" t="n">
-        <v>46214</v>
+        <v>46213</v>
       </c>
       <c r="B27" s="35" t="n">
         <v>4</v>
@@ -9497,7 +9497,7 @@
     </row>
     <row r="28">
       <c r="A28" s="106" t="n">
-        <v>46215</v>
+        <v>46214</v>
       </c>
       <c r="B28" s="35" t="n">
         <v>4</v>
@@ -9579,7 +9579,7 @@
     </row>
     <row r="29">
       <c r="A29" s="106" t="n">
-        <v>46216</v>
+        <v>46215</v>
       </c>
       <c r="B29" s="35" t="n">
         <v>4</v>
@@ -9665,7 +9665,7 @@
     </row>
     <row r="30">
       <c r="A30" s="106" t="n">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="B30" s="35" t="n">
         <v>4</v>
@@ -9747,7 +9747,7 @@
     </row>
     <row r="31">
       <c r="A31" s="106" t="n">
-        <v>46218</v>
+        <v>46217</v>
       </c>
       <c r="B31" s="35" t="n">
         <v>5</v>
@@ -9829,7 +9829,7 @@
     </row>
     <row r="32">
       <c r="A32" s="106" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="B32" s="35" t="n">
         <v>5</v>
@@ -9911,7 +9911,7 @@
     </row>
     <row r="33">
       <c r="A33" s="106" t="n">
-        <v>46220</v>
+        <v>46219</v>
       </c>
       <c r="B33" s="35" t="n">
         <v>5</v>
@@ -9993,7 +9993,7 @@
     </row>
     <row r="34">
       <c r="A34" s="106" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="B34" s="35" t="n">
         <v>5</v>
@@ -10075,7 +10075,7 @@
     </row>
     <row r="35">
       <c r="A35" s="106" t="n">
-        <v>46222</v>
+        <v>46221</v>
       </c>
       <c r="B35" s="35" t="n">
         <v>5</v>
@@ -10157,7 +10157,7 @@
     </row>
     <row r="36">
       <c r="A36" s="106" t="n">
-        <v>46223</v>
+        <v>46222</v>
       </c>
       <c r="B36" s="35" t="n">
         <v>5</v>
@@ -10243,7 +10243,7 @@
     </row>
     <row r="37">
       <c r="A37" s="106" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="B37" s="35" t="n">
         <v>5</v>
@@ -10325,7 +10325,7 @@
     </row>
     <row r="38">
       <c r="A38" s="106" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="B38" s="35" t="n">
         <v>6</v>
@@ -10407,7 +10407,7 @@
     </row>
     <row r="39">
       <c r="A39" s="106" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="B39" s="35" t="n">
         <v>6</v>
@@ -10489,7 +10489,7 @@
     </row>
     <row r="40">
       <c r="A40" s="106" t="n">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="B40" s="35" t="n">
         <v>6</v>
@@ -10571,7 +10571,7 @@
     </row>
     <row r="41">
       <c r="A41" s="106" t="n">
-        <v>46228</v>
+        <v>46227</v>
       </c>
       <c r="B41" s="35" t="n">
         <v>6</v>
@@ -10653,7 +10653,7 @@
     </row>
     <row r="42">
       <c r="A42" s="106" t="n">
-        <v>46229</v>
+        <v>46228</v>
       </c>
       <c r="B42" s="35" t="n">
         <v>6</v>
@@ -10735,7 +10735,7 @@
     </row>
     <row r="43">
       <c r="A43" s="106" t="n">
-        <v>46230</v>
+        <v>46229</v>
       </c>
       <c r="B43" s="35" t="n">
         <v>6</v>
@@ -10821,7 +10821,7 @@
     </row>
     <row r="44">
       <c r="A44" s="106" t="n">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="B44" s="35" t="n">
         <v>6</v>
@@ -10903,7 +10903,7 @@
     </row>
     <row r="45">
       <c r="A45" s="106" t="n">
-        <v>46232</v>
+        <v>46231</v>
       </c>
       <c r="B45" s="35" t="n">
         <v>7</v>
@@ -10985,7 +10985,7 @@
     </row>
     <row r="46">
       <c r="A46" s="106" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="B46" s="35" t="n">
         <v>7</v>
@@ -11067,7 +11067,7 @@
     </row>
     <row r="47">
       <c r="A47" s="106" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="B47" s="35" t="n">
         <v>7</v>
@@ -11149,7 +11149,7 @@
     </row>
     <row r="48">
       <c r="A48" s="106" t="n">
-        <v>46235</v>
+        <v>46234</v>
       </c>
       <c r="B48" s="35" t="n">
         <v>7</v>
@@ -11231,7 +11231,7 @@
     </row>
     <row r="49">
       <c r="A49" s="106" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B49" s="35" t="n">
         <v>7</v>
@@ -11313,7 +11313,7 @@
     </row>
     <row r="50">
       <c r="A50" s="106" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B50" s="35" t="n">
         <v>7</v>
@@ -11399,7 +11399,7 @@
     </row>
     <row r="51">
       <c r="A51" s="106" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="B51" s="35" t="n">
         <v>7</v>
@@ -11481,7 +11481,7 @@
     </row>
     <row r="52">
       <c r="A52" s="106" t="n">
-        <v>46239</v>
+        <v>46238</v>
       </c>
       <c r="B52" s="35" t="n">
         <v>8</v>
@@ -11563,7 +11563,7 @@
     </row>
     <row r="53">
       <c r="A53" s="106" t="n">
-        <v>46240</v>
+        <v>46239</v>
       </c>
       <c r="B53" s="35" t="n">
         <v>8</v>
@@ -11645,7 +11645,7 @@
     </row>
     <row r="54">
       <c r="A54" s="106" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="B54" s="35" t="n">
         <v>8</v>
@@ -11727,7 +11727,7 @@
     </row>
     <row r="55">
       <c r="A55" s="106" t="n">
-        <v>46242</v>
+        <v>46241</v>
       </c>
       <c r="B55" s="35" t="n">
         <v>8</v>
@@ -11809,7 +11809,7 @@
     </row>
     <row r="56">
       <c r="A56" s="106" t="n">
-        <v>46243</v>
+        <v>46242</v>
       </c>
       <c r="B56" s="35" t="n">
         <v>8</v>
@@ -11891,7 +11891,7 @@
     </row>
     <row r="57">
       <c r="A57" s="106" t="n">
-        <v>46244</v>
+        <v>46243</v>
       </c>
       <c r="B57" s="35" t="n">
         <v>8</v>
@@ -11977,7 +11977,7 @@
     </row>
     <row r="58">
       <c r="A58" s="106" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="B58" s="35" t="n">
         <v>8</v>
@@ -13530,11 +13530,11 @@
     </row>
     <row r="3">
       <c r="A3" s="106" t="n">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="B3" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C3" s="104" t="str"/>
@@ -13557,11 +13557,11 @@
     </row>
     <row r="4">
       <c r="A4" s="106" t="n">
-        <v>46191</v>
+        <v>46190</v>
       </c>
       <c r="B4" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C4" s="104" t="str"/>
@@ -13584,11 +13584,11 @@
     </row>
     <row r="5">
       <c r="A5" s="106" t="n">
-        <v>46192</v>
+        <v>46191</v>
       </c>
       <c r="B5" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C5" s="104" t="str"/>
@@ -13611,11 +13611,11 @@
     </row>
     <row r="6">
       <c r="A6" s="106" t="n">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C6" s="104" t="str"/>
@@ -13638,11 +13638,11 @@
     </row>
     <row r="7">
       <c r="A7" s="106" t="n">
-        <v>46194</v>
+        <v>46193</v>
       </c>
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C7" s="104" t="str"/>
@@ -13665,11 +13665,11 @@
     </row>
     <row r="8">
       <c r="A8" s="106" t="n">
-        <v>46195</v>
+        <v>46194</v>
       </c>
       <c r="B8" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C8" s="104" t="str"/>
@@ -13692,11 +13692,11 @@
     </row>
     <row r="9">
       <c r="A9" s="106" t="n">
-        <v>46196</v>
+        <v>46195</v>
       </c>
       <c r="B9" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C9" s="104" t="str"/>
@@ -13719,11 +13719,11 @@
     </row>
     <row r="10">
       <c r="A10" s="106" t="n">
-        <v>46197</v>
+        <v>46196</v>
       </c>
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C10" s="104" t="str"/>
@@ -13746,11 +13746,11 @@
     </row>
     <row r="11">
       <c r="A11" s="106" t="n">
-        <v>46198</v>
+        <v>46197</v>
       </c>
       <c r="B11" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C11" s="104" t="str"/>
@@ -13773,11 +13773,11 @@
     </row>
     <row r="12">
       <c r="A12" s="106" t="n">
-        <v>46199</v>
+        <v>46198</v>
       </c>
       <c r="B12" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C12" s="104" t="str"/>
@@ -13800,11 +13800,11 @@
     </row>
     <row r="13">
       <c r="A13" s="106" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C13" s="104" t="str"/>
@@ -13827,11 +13827,11 @@
     </row>
     <row r="14">
       <c r="A14" s="106" t="n">
-        <v>46201</v>
+        <v>46200</v>
       </c>
       <c r="B14" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C14" s="104" t="str"/>
@@ -13854,11 +13854,11 @@
     </row>
     <row r="15">
       <c r="A15" s="106" t="n">
-        <v>46202</v>
+        <v>46201</v>
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C15" s="104" t="str"/>
@@ -13881,11 +13881,11 @@
     </row>
     <row r="16">
       <c r="A16" s="106" t="n">
-        <v>46203</v>
+        <v>46202</v>
       </c>
       <c r="B16" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C16" s="104" t="str"/>
@@ -13908,11 +13908,11 @@
     </row>
     <row r="17">
       <c r="A17" s="106" t="n">
-        <v>46204</v>
+        <v>46203</v>
       </c>
       <c r="B17" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C17" s="104" t="str"/>
@@ -13935,11 +13935,11 @@
     </row>
     <row r="18">
       <c r="A18" s="106" t="n">
-        <v>46205</v>
+        <v>46204</v>
       </c>
       <c r="B18" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C18" s="104" t="str"/>
@@ -13962,11 +13962,11 @@
     </row>
     <row r="19">
       <c r="A19" s="106" t="n">
-        <v>46206</v>
+        <v>46205</v>
       </c>
       <c r="B19" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C19" s="104" t="str"/>
@@ -13989,11 +13989,11 @@
     </row>
     <row r="20">
       <c r="A20" s="106" t="n">
-        <v>46207</v>
+        <v>46206</v>
       </c>
       <c r="B20" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C20" s="104" t="str"/>
@@ -14016,11 +14016,11 @@
     </row>
     <row r="21">
       <c r="A21" s="106" t="n">
-        <v>46208</v>
+        <v>46207</v>
       </c>
       <c r="B21" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C21" s="104" t="str"/>
@@ -14043,11 +14043,11 @@
     </row>
     <row r="22">
       <c r="A22" s="106" t="n">
-        <v>46209</v>
+        <v>46208</v>
       </c>
       <c r="B22" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C22" s="104" t="str"/>
@@ -14070,11 +14070,11 @@
     </row>
     <row r="23">
       <c r="A23" s="106" t="n">
-        <v>46210</v>
+        <v>46209</v>
       </c>
       <c r="B23" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C23" s="104" t="str"/>
@@ -14097,11 +14097,11 @@
     </row>
     <row r="24">
       <c r="A24" s="106" t="n">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="B24" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C24" s="104" t="str"/>
@@ -14124,11 +14124,11 @@
     </row>
     <row r="25">
       <c r="A25" s="106" t="n">
-        <v>46212</v>
+        <v>46211</v>
       </c>
       <c r="B25" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C25" s="104" t="str"/>
@@ -14151,11 +14151,11 @@
     </row>
     <row r="26">
       <c r="A26" s="106" t="n">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="B26" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C26" s="104" t="str"/>
@@ -14178,11 +14178,11 @@
     </row>
     <row r="27">
       <c r="A27" s="106" t="n">
-        <v>46214</v>
+        <v>46213</v>
       </c>
       <c r="B27" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C27" s="104" t="str"/>
@@ -14205,11 +14205,11 @@
     </row>
     <row r="28">
       <c r="A28" s="106" t="n">
-        <v>46215</v>
+        <v>46214</v>
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C28" s="104" t="str"/>
@@ -14232,11 +14232,11 @@
     </row>
     <row r="29">
       <c r="A29" s="106" t="n">
-        <v>46216</v>
+        <v>46215</v>
       </c>
       <c r="B29" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C29" s="104" t="str"/>
@@ -14259,11 +14259,11 @@
     </row>
     <row r="30">
       <c r="A30" s="106" t="n">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C30" s="104" t="str"/>
@@ -14286,11 +14286,11 @@
     </row>
     <row r="31">
       <c r="A31" s="106" t="n">
-        <v>46218</v>
+        <v>46217</v>
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C31" s="104" t="str"/>
@@ -14313,11 +14313,11 @@
     </row>
     <row r="32">
       <c r="A32" s="106" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C32" s="104" t="str"/>
@@ -14340,11 +14340,11 @@
     </row>
     <row r="33">
       <c r="A33" s="106" t="n">
-        <v>46220</v>
+        <v>46219</v>
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C33" s="104" t="str"/>
@@ -14367,11 +14367,11 @@
     </row>
     <row r="34">
       <c r="A34" s="106" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C34" s="104" t="str"/>
@@ -14394,11 +14394,11 @@
     </row>
     <row r="35">
       <c r="A35" s="106" t="n">
-        <v>46222</v>
+        <v>46221</v>
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C35" s="104" t="str"/>
@@ -14421,11 +14421,11 @@
     </row>
     <row r="36">
       <c r="A36" s="106" t="n">
-        <v>46223</v>
+        <v>46222</v>
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C36" s="104" t="str"/>
@@ -14448,11 +14448,11 @@
     </row>
     <row r="37">
       <c r="A37" s="106" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C37" s="104" t="str"/>
@@ -14475,11 +14475,11 @@
     </row>
     <row r="38">
       <c r="A38" s="106" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C38" s="104" t="str"/>
@@ -14502,11 +14502,11 @@
     </row>
     <row r="39">
       <c r="A39" s="106" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C39" s="104" t="str"/>
@@ -14529,11 +14529,11 @@
     </row>
     <row r="40">
       <c r="A40" s="106" t="n">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C40" s="104" t="str"/>
@@ -14556,11 +14556,11 @@
     </row>
     <row r="41">
       <c r="A41" s="106" t="n">
-        <v>46228</v>
+        <v>46227</v>
       </c>
       <c r="B41" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C41" s="104" t="str"/>
@@ -14583,11 +14583,11 @@
     </row>
     <row r="42">
       <c r="A42" s="106" t="n">
-        <v>46229</v>
+        <v>46228</v>
       </c>
       <c r="B42" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C42" s="104" t="str"/>
@@ -14610,11 +14610,11 @@
     </row>
     <row r="43">
       <c r="A43" s="106" t="n">
-        <v>46230</v>
+        <v>46229</v>
       </c>
       <c r="B43" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C43" s="104" t="str"/>
@@ -14637,11 +14637,11 @@
     </row>
     <row r="44">
       <c r="A44" s="106" t="n">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="B44" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C44" s="104" t="str"/>
@@ -14664,11 +14664,11 @@
     </row>
     <row r="45">
       <c r="A45" s="106" t="n">
-        <v>46232</v>
+        <v>46231</v>
       </c>
       <c r="B45" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C45" s="104" t="str"/>
@@ -14691,11 +14691,11 @@
     </row>
     <row r="46">
       <c r="A46" s="106" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="B46" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C46" s="104" t="str"/>
@@ -14718,11 +14718,11 @@
     </row>
     <row r="47">
       <c r="A47" s="106" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="B47" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C47" s="104" t="str"/>
@@ -14745,11 +14745,11 @@
     </row>
     <row r="48">
       <c r="A48" s="106" t="n">
-        <v>46235</v>
+        <v>46234</v>
       </c>
       <c r="B48" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C48" s="104" t="str"/>
@@ -14772,11 +14772,11 @@
     </row>
     <row r="49">
       <c r="A49" s="106" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B49" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C49" s="104" t="str"/>
@@ -14799,11 +14799,11 @@
     </row>
     <row r="50">
       <c r="A50" s="106" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B50" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C50" s="104" t="str"/>
@@ -14826,11 +14826,11 @@
     </row>
     <row r="51">
       <c r="A51" s="106" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="B51" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C51" s="104" t="str"/>
@@ -14853,11 +14853,11 @@
     </row>
     <row r="52">
       <c r="A52" s="106" t="n">
-        <v>46239</v>
+        <v>46238</v>
       </c>
       <c r="B52" s="35" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C52" s="104" t="str"/>
@@ -14880,11 +14880,11 @@
     </row>
     <row r="53">
       <c r="A53" s="106" t="n">
-        <v>46240</v>
+        <v>46239</v>
       </c>
       <c r="B53" s="35" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C53" s="104" t="str"/>
@@ -14907,11 +14907,11 @@
     </row>
     <row r="54">
       <c r="A54" s="106" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="B54" s="35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C54" s="104" t="str"/>
@@ -14934,11 +14934,11 @@
     </row>
     <row r="55">
       <c r="A55" s="106" t="n">
-        <v>46242</v>
+        <v>46241</v>
       </c>
       <c r="B55" s="35" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C55" s="104" t="str"/>
@@ -14961,11 +14961,11 @@
     </row>
     <row r="56">
       <c r="A56" s="106" t="n">
-        <v>46243</v>
+        <v>46242</v>
       </c>
       <c r="B56" s="35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C56" s="104" t="str"/>
@@ -14988,11 +14988,11 @@
     </row>
     <row r="57">
       <c r="A57" s="106" t="n">
-        <v>46244</v>
+        <v>46243</v>
       </c>
       <c r="B57" s="35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C57" s="104" t="str"/>
@@ -15015,11 +15015,11 @@
     </row>
     <row r="58">
       <c r="A58" s="106" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="B58" s="35" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C58" s="104" t="str"/>

</xml_diff>

<commit_message>
Legs A: fix duplicate Leg Press (#1 → Hack Squat) + "45°" typo
#1 was "Hack Squat or Leg Press" while #3 was "Leg Press" — same machine
twice. #1 is now just Hack Squat (Leg Press stays at #3), so the day is two
distinct quad compounds + hinge + ham curl + quad ext + calves + core.
Also fixed "45– Back Extension" → "45° Back Extension". Applied to data.js
and the xlsx. Audited all other days: no duplicates.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Armen_2_Month_Gym_Meal_Plan_With_Timing.xlsx
+++ b/Armen_2_Month_Gym_Meal_Plan_With_Timing.xlsx
@@ -995,7 +995,6 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="33" t="inlineStr">
         <is>
@@ -1178,7 +1177,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="33" t="inlineStr">
         <is>
@@ -1539,8 +1537,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="33" t="inlineStr">
         <is>
@@ -5135,7 +5131,7 @@
       </c>
       <c r="C17" s="35" t="inlineStr">
         <is>
-          <t>Hack Squat or Leg Press</t>
+          <t>Hack Squat</t>
         </is>
       </c>
       <c r="D17" s="35" t="inlineStr">
@@ -5170,7 +5166,7 @@
       </c>
       <c r="J17" s="35" t="inlineStr">
         <is>
-          <t>Smith-machine squat or pendulum squat</t>
+          <t>Leg press, Smith-machine squat, or pendulum squat</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5181,7 @@
       </c>
       <c r="C18" s="35" t="inlineStr">
         <is>
-          <t>45– Back Extension (Hyperextension)</t>
+          <t>45° Back Extension (Hyperextension)</t>
         </is>
       </c>
       <c r="D18" s="35" t="inlineStr">
@@ -5270,7 +5266,7 @@
       </c>
       <c r="J19" s="35" t="inlineStr">
         <is>
-          <t>Hack squat</t>
+          <t>Pendulum squat or belt squat</t>
         </is>
       </c>
     </row>
@@ -6524,6 +6520,21 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
     <row r="60">
       <c r="A60" s="33" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Lower B: swap 3 exercises + fix sync dropping unsynced changes
Training:
- Hip Thrust (heavy) -> Heavy Leg Press
- Cable Pull-Through -> Cable/Machine Glute Kickback
- Core Circuit -> Hanging Leg Raise
Same Template#Order keys so logged weights are preserved; updated the
suggested starting weights and the source xlsx to match.

Sync (firebase-sync.js):
- Persist a device-local "pending" flag the moment a change is made, so a
  change made before sync is ready (or right before the tab closes) is no
  longer silently dropped.
- Flush pending changes on becoming ready and on visibilitychange/pagehide.
- On load, a device with unsynced local changes pushes them up instead of
  being overwritten by the cloud copy.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Armen_2_Month_Gym_Meal_Plan_With_Timing.xlsx
+++ b/Armen_2_Month_Gym_Meal_Plan_With_Timing.xlsx
@@ -5831,27 +5831,27 @@
       </c>
       <c r="C31" s="35" t="inlineStr">
         <is>
-          <t>Barbell or Machine Hip Thrust (heavy)</t>
+          <t>Heavy Leg Press</t>
         </is>
       </c>
       <c r="D31" s="35" t="inlineStr">
         <is>
-          <t>3 x 5 @ RPE 6–7</t>
+          <t>3 x 6 @ RPE 6–7</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>3 x 5 @ RPE 7–8</t>
+          <t>3 x 6 @ RPE 7–8</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>4 x 4–5 @ RPE 8</t>
+          <t>4 x 5–6 @ RPE 8</t>
         </is>
       </c>
       <c r="G31" s="35" t="inlineStr">
         <is>
-          <t>3 x 4–5</t>
+          <t>3 x 5–6</t>
         </is>
       </c>
       <c r="H31" s="35" t="inlineStr">
@@ -5861,12 +5861,12 @@
       </c>
       <c r="I31" s="35" t="inlineStr">
         <is>
-          <t>Drive through heels; ribs down; pause hard at top</t>
+          <t>Feet mid-platform; deep but controlled; drive through heels; don't slam-lock knees</t>
         </is>
       </c>
       <c r="J31" s="35" t="inlineStr">
         <is>
-          <t>Glute bridge machine or hip-thrust machine</t>
+          <t>Hack squat</t>
         </is>
       </c>
     </row>
@@ -5981,42 +5981,42 @@
       </c>
       <c r="C34" s="35" t="inlineStr">
         <is>
-          <t>Cable Pull-Through</t>
+          <t>Cable/Machine Glute Kickback</t>
         </is>
       </c>
       <c r="D34" s="35" t="inlineStr">
         <is>
-          <t>3 x 10</t>
+          <t>3 x 12/side</t>
         </is>
       </c>
       <c r="E34" s="35" t="inlineStr">
         <is>
-          <t>3 x 8–10</t>
+          <t>3 x 10–12/side</t>
         </is>
       </c>
       <c r="F34" s="35" t="inlineStr">
         <is>
-          <t>4 x 8–10</t>
+          <t>4 x 10–12/side</t>
         </is>
       </c>
       <c r="G34" s="35" t="inlineStr">
         <is>
-          <t>3 x 10</t>
+          <t>3 x 12/side</t>
         </is>
       </c>
       <c r="H34" s="35" t="inlineStr">
         <is>
-          <t>90 sec</t>
+          <t>60 sec</t>
         </is>
       </c>
       <c r="I34" s="35" t="inlineStr">
         <is>
-          <t>Hinge at hips; finish with glute squeeze, not lower back</t>
+          <t>Squeeze glute at top; no lower-back arch; control the return</t>
         </is>
       </c>
       <c r="J34" s="35" t="inlineStr">
         <is>
-          <t>45– back extension</t>
+          <t>Hip abduction machine</t>
         </is>
       </c>
     </row>
@@ -6131,27 +6131,27 @@
       </c>
       <c r="C37" s="35" t="inlineStr">
         <is>
-          <t>Core Circuit: Cable Crunch, Side Plank, Dead Bug</t>
+          <t>Hanging Leg Raise</t>
         </is>
       </c>
       <c r="D37" s="35" t="inlineStr">
         <is>
-          <t>2 rounds</t>
+          <t>3 x 10</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>3 rounds</t>
+          <t>3 x 10–12</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>3–4 rounds</t>
+          <t>3–4 x 10–12</t>
         </is>
       </c>
       <c r="G37" s="35" t="inlineStr">
         <is>
-          <t>3 rounds</t>
+          <t>3 x 12</t>
         </is>
       </c>
       <c r="H37" s="35" t="inlineStr">
@@ -6161,12 +6161,12 @@
       </c>
       <c r="I37" s="35" t="inlineStr">
         <is>
-          <t>Control breathing</t>
+          <t>No swinging; curl pelvis toward ribs; lower slow</t>
         </is>
       </c>
       <c r="J37" s="35" t="inlineStr">
         <is>
-          <t>Ab machine</t>
+          <t>Captain's chair knee raise</t>
         </is>
       </c>
     </row>
@@ -6520,21 +6520,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="33" t="inlineStr">
         <is>

</xml_diff>